<commit_message>
Model: add per-order cost (23 UAH) and upsell commission (23%), UA ad counts for candidates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016SrNoYKzYt6F2gDAr7eBJZ
</commit_message>
<xml_diff>
--- a/model/Product_Hunter_Model.xlsx
+++ b/model/Product_Hunter_Model.xlsx
@@ -682,7 +682,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Апрув 64 % і викуп 82 % — ваші середні цифри. Конкретні значення по кожному товару підставимо з LP-CRM.</t>
+          <t>• Апрув 64 %, викуп 82 %, 23 ₴ витрат на замовлення і 23 % комісії з допродажів — ваші цифри; повернення невикупу 100 ₴ — припущення. Конкретні значення по кожному товару підставимо з LP-CRM.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -821,15 +821,15 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Інші витрати на 1 підтверджене замовлення (кол-центр, пакування), ₴</t>
+          <t>Інші витрати на 1 підтверджене замовлення, ₴</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>ЗАПОВНІТЬ: зараз 0, тому прибуток завищений</t>
+          <t>Від користувача: 23 ₴ за підтверджене замовлення</t>
         </is>
       </c>
     </row>
@@ -935,6 +935,21 @@
       <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Рішення про стоп після спенду = N × цільовий CPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Комісія з маржі допродажів</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Від користувача: 23 % з маржі допродажів</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1030,12 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>Параметри!B4+Параметри!B5</f>
+        <f>Параметри!B4+Параметри!B5*(1-Параметри!B17)</f>
         <v/>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>маржа товару + допродажі</t>
+          <t>маржа товару + допродажі мінус комісія з допродажів</t>
         </is>
       </c>
       <c r="D4" s="5" t="n"/>
@@ -2474,7 +2489,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>92 активні оголошення US; біль «прибирання без нахилів»</t>
+          <t>US: 92 активні оголошення; UA: ~95 (частина нерелевантні); біль «прибирання без нахилів»</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2541,7 @@
       </c>
       <c r="N6" s="20" t="inlineStr">
         <is>
-          <t>105 оголошень US, тренд TikTok Shop; ваш вакууматор мав CPL $4.4 (мала вибірка)</t>
+          <t>US: 105 оголошень, тренд TikTok Shop; UA: ~115; ваш вакууматор мав CPL $4.4 (мала вибірка)</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2593,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>556 оголошень US, багато клонів; низький чек — краще як допродаж</t>
+          <t>US: 556 оголошень, багато клонів; UA «подрібнювач»: ~169; низький чек — краще як допродаж</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Model: set return cost to 150 UAH per user
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016SrNoYKzYt6F2gDAr7eBJZ
</commit_message>
<xml_diff>
--- a/model/Product_Hunter_Model.xlsx
+++ b/model/Product_Hunter_Model.xlsx
@@ -682,7 +682,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Апрув 64 %, викуп 82 %, 23 ₴ витрат на замовлення і 23 % комісії з допродажів — ваші цифри; повернення невикупу 100 ₴ — припущення. Конкретні значення по кожному товару підставимо з LP-CRM.</t>
+          <t>• Апрув 64 %, викуп 82 %, 23 ₴ витрат на замовлення і 23 % комісії з допродажів — ваші цифри; повернення невикупу ~150 ₴. Конкретні значення по кожному товару підставимо з LP-CRM.</t>
         </is>
       </c>
     </row>
@@ -810,11 +810,11 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ПРИПУЩЕННЯ: зворотна доставка ~100 ₴. Уточніть</t>
+          <t>Від користувача: ~150 ₴</t>
         </is>
       </c>
     </row>

</xml_diff>